<commit_message>
Update outreach pitches for leads without website with dual demo links and add pitch modal to dashboard
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -513,7 +513,7 @@
     <col width="17" customWidth="1" min="38" max="38"/>
     <col width="40" customWidth="1" min="39" max="39"/>
     <col width="40" customWidth="1" min="40" max="40"/>
-    <col width="37" customWidth="1" min="41" max="41"/>
+    <col width="40" customWidth="1" min="41" max="41"/>
     <col width="22" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
@@ -804,7 +804,7 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917086547703?text=Hi%20from%20Atrya%20Solutions%21%20%0A%0AWe%20help%20CCTV%20companies%20like%20Beast%20Sound%20Installations%20get%20direct%20customers.%20%0A%0AImagine%20capturing%20Google%20leads%20instantly%20with%20a%20professional%20website%20and%201-click%20WhatsApp%20quotes%2C%20instead%20of%20relying%20on%20Justdial%20commissions.%20%0A%0ASee%20a%20DEMO%20of%20what%20we%20customize%20and%20build%20for%20CCTV%20businesses%3A%20https%3A//atryasolutions.netlify.app/%0A%0AWould%20you%20be%20open%20to%20a%2015-minute%20walkthrough%3F</t>
+          <t>https://wa.me/917086547703?text=Hi%20Beast%20Sound%20Installations%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr"/>
@@ -882,24 +882,33 @@
       <c r="AL2" s="2" t="inlineStr"/>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>Hi from Atrya Solutions! 
-We help CCTV companies like Beast Sound Installations get direct customers. 
-Imagine capturing Google leads instantly with a professional website and 1-click WhatsApp quotes, instead of relying on Justdial commissions. 
-See a DEMO of what we customize and build for CCTV businesses: https://atryasolutions.netlify.app/
-Would you be open to a 15-minute walkthrough?</t>
+          <t>Hi Beast Sound Installations,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>Boost Direct Leads: Beast Sound Installations</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Beast Sound Installations</t>
         </is>
       </c>
       <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>Hi Beast Sound Installations Team,
-Atrya Solutions builds high-converting websites for CCTV companies. We noticed you're missing an official website, potentially losing direct Google customers to commission-based platforms.
-Our professional sites feature instant 1-click WhatsApp quote buttons, designed to capture leads directly. See a DEMO of what we customize: https://atryasolutions.netlify.app/
-Let's connect for a 15-minute walkthrough to show you how we can help you get more direct enquiries.
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -984,7 +993,7 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
-          <t>https://wa.me/917733893955?text=Hi%20NC%20Security%20System%2C%0A%0AI%20noticed%20you%20don%E2%80%99t%20have%20a%20website%20yet.%20A%20custom%20lead%E2%80%91gen%20site%20with%20instant%201%E2%80%91click%20WhatsApp%20quote%20can%20pull%20Google%20customers%20directly%2C%20saving%20you%20Justdial%20fees.%0A%0ACan%20we%20schedule%20a%2015%E2%80%91min%20walkthrough%20of%20our%20demo%3F%0A%0ABest%2C%0A%5BYour%20Name%5D</t>
+          <t>https://wa.me/917733893955?text=Hi%20NC%20Security%20System%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R3" s="4" t="inlineStr"/>
@@ -1055,23 +1064,32 @@
       <c r="AM3" s="4" t="inlineStr">
         <is>
           <t>Hi NC Security System,
-I noticed you don’t have a website yet. A custom lead‑gen site with instant 1‑click WhatsApp quote can pull Google customers directly, saving you Justdial fees.
-Can we schedule a 15‑min walkthrough of our demo?
-Best,
-[Your Name]</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN3" s="4" t="inlineStr">
         <is>
-          <t>Get Direct Google Leads, No Website Needed</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for NC Security System</t>
         </is>
       </c>
       <c r="AO3" s="4" t="inlineStr">
         <is>
-          <t>Hi NC Security System,
-I see you currently rely on directories and social media without an official website. That means you’re paying commissions to platforms like Justdial while missing out on direct Google traffic.
-A tailored, SEO‑optimized website with instant 1‑click WhatsApp quote buttons can capture those high‑intent customers and route them straight to you, eliminating third‑party fees.
-We’d love to show you a quick 15‑minute walkthrough of our live demo and discuss how it can boost your lead flow.
+          <t>Hi NC Security System Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -1156,7 +1174,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917735058027?text=Hi%20Protal247%2C%0AI%20noticed%20you%20don%E2%80%99t%20have%20a%20website%2C%20so%20you%E2%80%99re%20likely%20paying%20commissions%20on%20Justdial%20for%20leads.%20We%20build%20high%E2%80%91converting%20lead%E2%80%91gen%20sites%20with%20instant%201%E2%80%91click%20WhatsApp%20quote%20buttons%2C%20driving%20direct%20Google%20customers.%0ACan%20we%20schedule%20a%2015%E2%80%91min%20walkthrough%3F%20Demo%3A%20https%3A//atryasolutions.netlify.app/</t>
+          <t>https://wa.me/917735058027?text=Hi%20Protal247%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr"/>
@@ -1227,21 +1245,32 @@
       <c r="AM4" s="2" t="inlineStr">
         <is>
           <t>Hi Protal247,
-I noticed you don’t have a website, so you’re likely paying commissions on Justdial for leads. We build high‑converting lead‑gen sites with instant 1‑click WhatsApp quote buttons, driving direct Google customers.
-Can we schedule a 15‑min walkthrough? Demo: https://atryasolutions.netlify.app/</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>Stop Paying Lead Commissions</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Protal247</t>
         </is>
       </c>
       <c r="AO4" s="2" t="inlineStr">
         <is>
-          <t>Hi [Name],
-I see Protal247 currently relies on directories for leads, which means you’re paying commissions on every enquiry. A custom, SEO‑optimized website with a 1‑click WhatsApp quote button can capture direct Google customers, eliminating those fees and boosting conversion rates.
-We’ve built similar solutions for CCTV firms—see our DEMO site (https://atryasolutions.netlify.app/). The platform also integrates a powerful admin panel for job tracking and AMC dispatch, should you need it later.
-Would a 15‑minute walkthrough this week work for you?
+          <t>Hi Protal247 Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -1326,7 +1355,7 @@
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>https://wa.me/917733457641?text=Hi%20from%20Atrya%20Solutions%21%0A%0AImagine%20getting%20direct%20customer%20calls%20from%20Google%2C%20not%20just%20Justdial.%0A%0AWe%20build%20professional%20websites%20for%20CCTV%20%26%20security%20companies%20like%20yours%20to%20capture%20local%20leads%20directly.%0A%0ABoost%20your%20business%20without%20paying%20commissions.%20Let%27s%20chat%20for%2015%20mins%3F</t>
+          <t>https://wa.me/917733457641?text=Hi%20Premier%20Intercom%20Installation%2C%20Repair%20Services%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R5" s="4" t="inlineStr"/>
@@ -1396,24 +1425,33 @@
       <c r="AL5" s="4" t="inlineStr"/>
       <c r="AM5" s="4" t="inlineStr">
         <is>
-          <t>Hi from Atrya Solutions!
-Imagine getting direct customer calls from Google, not just Justdial.
-We build professional websites for CCTV &amp; security companies like yours to capture local leads directly.
-Boost your business without paying commissions. Let's chat for 15 mins?</t>
+          <t>Hi Premier Intercom Installation, Repair Services,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN5" s="4" t="inlineStr">
         <is>
-          <t>Stop Paying Justdial Commissions?</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Premier Intercom Installation, Repair Services</t>
         </is>
       </c>
       <c r="AO5" s="4" t="inlineStr">
         <is>
-          <t>Hello Premier Intercom Team,
-Are you tired of relying solely on directories like Justdial and paying high commissions for leads?
-At Atrya Solutions, we specialize in building high-converting websites for CCTV and electronic security companies. Our sites are designed to capture direct customer inquiries from Google, helping you grow your business more profitably.
-See a demo of what we customize and build for businesses like yours: https://atryasolutions.netlify.app/
-Would you be open to a quick 15-minute walkthrough to show you how we can help you get direct customers?
+          <t>Hi Premier Intercom Installation, Repair Services Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -1498,7 +1536,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917085951156?text=Hi%20Video%E2%80%91Comm%2C%0AI%20noticed%20you%20don%E2%80%99t%20have%20a%20website%2C%20so%20you%E2%80%99re%20missing%20direct%20Google%20leads%20and%20paying%20commissions%20on%20directories.%20We%20build%20high%E2%80%91converting%20sites%20with%20instant%201%E2%80%91click%20WhatsApp%20quote%20buttons%20that%20capture%20customers%20instantly.%0ACan%20we%20schedule%20a%2015%E2%80%91min%20walkthrough%3F%20%E2%80%93%20Atrya%20Solutions</t>
+          <t>https://wa.me/917085951156?text=Hi%20Video-Comm%20Security%20Cameras%202%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr"/>
@@ -1568,21 +1606,33 @@
       <c r="AL6" s="2" t="inlineStr"/>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>Hi Video‑Comm,
-I noticed you don’t have a website, so you’re missing direct Google leads and paying commissions on directories. We build high‑converting sites with instant 1‑click WhatsApp quote buttons that capture customers instantly.
-Can we schedule a 15‑min walkthrough? – Atrya Solutions</t>
+          <t>Hi Video-Comm Security Cameras 2,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>Capture Direct Google Leads</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Video-Comm Security Cameras 2</t>
         </is>
       </c>
       <c r="AO6" s="2" t="inlineStr">
         <is>
-          <t>Hi Video‑Comm Security Cameras 2,
-I saw you currently rely on directories and social media without an official website. That means you’re losing direct Google traffic and paying commissions to platforms like Justdial. At Atrya Solutions we create professional lead‑generation websites tailored for CCTV businesses, featuring instant 1‑click WhatsApp quote buttons that turn visitors into qualified leads instantly.
-We’d love to show you a quick 15‑minute walkthrough of our demo and discuss how a custom site can start driving customers straight from Google.
+          <t>Hi Video-Comm Security Cameras 2 Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -1667,7 +1717,7 @@
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>https://wa.me/919178325446?text=Hi%20InstallTech%2C%20I%27m%20%5BYour%20Name%5D%20from%20Atrya%20Solutions.%0A%0AWe%20build%20websites%20specifically%20for%20security%20companies%20like%20yours%20to%20capture%20direct%20customers%20from%20Google.%0A%0AImagine%20getting%20leads%20without%20paying%20commissions%20to%20Justdial%20or%20other%20directories.%20Our%20sites%20feature%20instant%20WhatsApp%20quote%20buttons.%0A%0AWould%20you%20be%20open%20to%20a%20quick%2015-minute%20demo%20of%20what%20we%20customize%20and%20build%3F</t>
+          <t>https://wa.me/919178325446?text=Hi%20InstallTech.%20Security%20Camera%20Systems.%20Data%26Telecom.%20INC%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R7" s="4" t="inlineStr"/>
@@ -1737,24 +1787,33 @@
       <c r="AL7" s="4" t="inlineStr"/>
       <c r="AM7" s="4" t="inlineStr">
         <is>
-          <t>Hi InstallTech, I'm [Your Name] from Atrya Solutions.
-We build websites specifically for security companies like yours to capture direct customers from Google.
-Imagine getting leads without paying commissions to Justdial or other directories. Our sites feature instant WhatsApp quote buttons.
-Would you be open to a quick 15-minute demo of what we customize and build?</t>
+          <t>Hi InstallTech. Security Camera Systems. Data&amp;Telecom. INC,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN7" s="4" t="inlineStr">
         <is>
-          <t>Stop Paying Commissions: Get Direct Leads</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for InstallTech. Security Camera Systems. Data&amp;Telecom. INC</t>
         </is>
       </c>
       <c r="AO7" s="4" t="inlineStr">
         <is>
-          <t>Hi InstallTech Team,
-I noticed you're doing great work, but might be missing out on direct customer leads by not having an official website.
-Atrya Solutions specializes in building high-converting websites for security companies. Our sites help you capture direct customers from Google, reducing reliance on commission-based directories.
-We include features like 1-click WhatsApp quote buttons to boost inquiries.
-Would you be open to a 15-minute walkthrough of a demo we customize and build for businesses like yours?
+          <t>Hi InstallTech. Security Camera Systems. Data&amp;Telecom. INC Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -1839,7 +1898,7 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/918728069753?text=Hi%20%5BName%5D%2C%0AI%E2%80%99m%20from%20Atrya%20Solutions.%20We%20help%20CCTV%20firms%20capture%20direct%20Google%20leads%20with%20a%20high%E2%80%91converting%20website%20and%20instant%201%E2%80%91click%20WhatsApp%20quote%20button%E2%80%94no%20more%20paying%20Justdial%20commissions.%0ACan%20we%20schedule%20a%2015%E2%80%91min%20walkthrough%3F%20Demo%3A%20https%3A//atryasolutions.netlify.app/</t>
+          <t>https://wa.me/918728069753?text=Hi%20Security%20Cameras%20Solutions%20Geek%20Tech%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr"/>
@@ -1909,22 +1968,33 @@
       <c r="AL8" s="2" t="inlineStr"/>
       <c r="AM8" s="2" t="inlineStr">
         <is>
-          <t>Hi [Name],
-I’m from Atrya Solutions. We help CCTV firms capture direct Google leads with a high‑converting website and instant 1‑click WhatsApp quote button—no more paying Justdial commissions.
-Can we schedule a 15‑min walkthrough? Demo: https://atryasolutions.netlify.app/</t>
+          <t>Hi Security Cameras Solutions Geek Tech,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>Get Direct Google Leads Free</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Security Cameras Solutions Geek Tech</t>
         </is>
       </c>
       <c r="AO8" s="2" t="inlineStr">
         <is>
-          <t>Hi [First Name],
-I noticed Security Cameras Solutions Geek Tech doesn’t have an official website and relies on directories. That means you’re paying commissions on Justdial and missing out on direct Google customers.
-Atrya Solutions builds professional lead‑generation sites with instant 1‑click WhatsApp quote buttons, driving high‑quality enquiries straight from Google. We’ll handle the design, SEO and integration at no upfront cost, so you capture leads without third‑party fees.
-Would you be open to a 15‑minute walkthrough of our demo and discuss a free custom build? Demo: https://atryasolutions.netlify.app/
+          <t>Hi Security Cameras Solutions Geek Tech Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -2068,24 +2138,32 @@
       <c r="AM9" s="4" t="inlineStr">
         <is>
           <t>Hi Chicago Electrical Services,
-Imagine capturing direct Google customers instead of paying commissions.
-We build high-converting websites specifically for CCTV &amp; electronic security companies, featuring instant 1-click WhatsApp quotes.
-See a DEMO of what we customize: https://atryasolutions.netlify.app/
-Would you be open to a quick 15-minute walkthrough?</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN9" s="4" t="inlineStr">
         <is>
-          <t>Boost Leads: Your Direct Website Solution</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Chicago Electrical Services</t>
         </is>
       </c>
       <c r="AO9" s="4" t="inlineStr">
         <is>
-          <t>Dear Chicago Electrical Services,
-Are you tired of relying solely on directories and paying commissions for leads? We specialize in building professional, lead-generation websites for CCTV and electronic security businesses.
-Our sites feature instant 1-click WhatsApp quote buttons, designed to convert visitors into direct customers.
-See a DEMO of what we customize and build: https://atryasolutions.netlify.app/
-Let's connect for a brief 15-minute walkthrough to show you how we can help you capture more direct business.
+          <t>Hi Chicago Electrical Services Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -2170,7 +2248,7 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917736374422?text=Hi%20Detect%20All%20Security%2C%0A%0AI%20noticed%20you%20don%E2%80%99t%20have%20a%20website%2C%20so%20you%E2%80%99re%20missing%20direct%20Google%20leads%20and%20paying%20commissions%20on%20Justdial.%20We%20build%20high%E2%80%91converting%20sites%20with%20instant%201%E2%80%91click%20WhatsApp%20quote%20buttons%20%28demo%3A%20https%3A//atryasolutions.netlify.app/%29.%20Can%20we%20schedule%20a%2015%E2%80%91min%20walkthrough%3F%0A%0AReply%20STOP%20and%20I%20won%27t%20contact%20you%20again.</t>
+          <t>https://wa.me/917736374422?text=Hi%20Detect%20All%20Security%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr"/>
@@ -2241,19 +2319,32 @@
       <c r="AM10" s="2" t="inlineStr">
         <is>
           <t>Hi Detect All Security,
-I noticed you don’t have a website, so you’re missing direct Google leads and paying commissions on Justdial. We build high‑converting sites with instant 1‑click WhatsApp quote buttons (demo: https://atryasolutions.netlify.app/). Can we schedule a 15‑min walkthrough?
-Reply STOP and I won't contact you again.</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>Capture Direct Google Leads Today</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Detect All Security</t>
         </is>
       </c>
       <c r="AO10" s="2" t="inlineStr">
         <is>
-          <t>Hi [First Name],
-I see Detect All Security currently relies on directories and social media, missing out on direct Google traffic and paying commissions on platforms like Justdial. A custom, SEO‑optimized website with instant 1‑click WhatsApp quote buttons can turn searchers into qualified leads instantly. We’ve built similar solutions for CCTV firms—see our demo at https://atryasolutions.netlify.app/. I’d love to walk you through a 15‑minute, no‑obligation demo of how we can boost your lead flow and reduce third‑party costs.
+          <t>Hi Detect All Security Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -2393,24 +2484,32 @@
       <c r="AM11" s="4" t="inlineStr">
         <is>
           <t>Hi Electro Alarm Co Inc,
-Are you tired of relying on Justdial or IndiaMART for leads?
-We build professional websites that capture direct Google customers, complete with 1-click WhatsApp quote buttons. Imagine instant inquiries without commissions!
-See a DEMO of what we customize for CCTV businesses: https://atryasolutions.netlify.app/
-Let's chat for 15 mins?</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN11" s="4" t="inlineStr">
         <is>
-          <t>Stop Paying Commissions: Get Direct Leads</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Electro Alarm Co Inc</t>
         </is>
       </c>
       <c r="AO11" s="4" t="inlineStr">
         <is>
-          <t>Hi Electro Alarm Co Inc,
-Are you looking to capture more direct customers without paying hefty commissions to directories like Justdial?
-We specialize in building high-converting websites for CCTV businesses. Our sites feature instant 1-click WhatsApp quote buttons, designed to turn visitors into leads.
-See a DEMO of what we customize: https://atryasolutions.netlify.app/
-Would you be open to a quick 15-minute walkthrough to show you how we can help you get direct Google customers?
+          <t>Hi Electro Alarm Co Inc Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -2487,7 +2586,7 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/917083955335?text=Hi%2C%0AI%20noticed%20DVR%20USA%20Security%20has%20no%20official%20website%2C%20meaning%20you%E2%80%99re%20missing%20direct%20Google%20leads%20and%20still%20paying%20commissions%20on%20directories.%20We%20build%20high%E2%80%91converting%20lead%E2%80%91gen%20sites%20with%20instant%201%E2%80%91click%20WhatsApp%20quote%20buttons.%0ACan%20we%20schedule%20a%2015%E2%80%91minute%20walkthrough%3F%0AReply%20STOP%20to%20opt%E2%80%91out.</t>
+          <t>https://wa.me/917083955335?text=Hi%20DVR%20USA%20Security%20Inc%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr"/>
@@ -2557,26 +2656,33 @@
       <c r="AL12" s="2" t="inlineStr"/>
       <c r="AM12" s="2" t="inlineStr">
         <is>
-          <t>Hi,
-I noticed DVR USA Security has no official website, meaning you’re missing direct Google leads and still paying commissions on directories. We build high‑converting lead‑gen sites with instant 1‑click WhatsApp quote buttons.
-Can we schedule a 15‑minute walkthrough?
-Reply STOP to opt‑out.</t>
+          <t>Hi DVR USA Security Inc,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>Capture Direct Google Leads Now</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for DVR USA Security Inc</t>
         </is>
       </c>
       <c r="AO12" s="2" t="inlineStr">
         <is>
-          <t>Hello,
-I saw DVR USA Security currently relies only on directories and social media, with no dedicated website. That limits your ability to capture direct Google customers and forces you to pay commissions on platforms like Justdial.
-A professional, SEO‑optimized site with instant 1‑click WhatsApp quote buttons can turn search traffic into qualified leads instantly.
-We’d love to show you a quick 15‑minute walkthrough of a live demo tailored for CCTV businesses.
+          <t>Hi DVR USA Security Inc Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
 Best regards,
-[Your Name]
-Atrya Solutions
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -2653,7 +2759,7 @@
       </c>
       <c r="Q13" s="5" t="inlineStr">
         <is>
-          <t>https://wa.me/918154355200?text=Hi%20from%20Atrya%20Solutions%21%0A%0AImagine%20getting%20direct%20customer%20leads%20from%20Google%2C%20instead%20of%20paying%20high%20commissions%20to%20Justdial.%0A%0AWe%20build%20professional%20websites%20with%201-click%20WhatsApp%20quotes%2C%20customized%20for%20CCTV%20businesses.%0A%0ASee%20a%20DEMO%20of%20what%20we%20build%3A%20https%3A//atryasolutions.netlify.app/%0A%0ABook%20a%2015-min%20walkthrough%20to%20see%20how%20we%20can%20help%20Home%20Security%20Direct%20grow.</t>
+          <t>https://wa.me/918154355200?text=Hi%20Home%20Security%20Direct%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R13" s="4" t="inlineStr"/>
@@ -2723,26 +2829,33 @@
       <c r="AL13" s="4" t="inlineStr"/>
       <c r="AM13" s="4" t="inlineStr">
         <is>
-          <t>Hi from Atrya Solutions!
-Imagine getting direct customer leads from Google, instead of paying high commissions to Justdial.
-We build professional websites with 1-click WhatsApp quotes, customized for CCTV businesses.
-See a DEMO of what we build: https://atryasolutions.netlify.app/
-Book a 15-min walkthrough to see how we can help Home Security Direct grow.</t>
+          <t>Hi Home Security Direct,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN13" s="4" t="inlineStr">
         <is>
-          <t>Stop Paying Justdial Commissions?</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Home Security Direct</t>
         </is>
       </c>
       <c r="AO13" s="4" t="inlineStr">
         <is>
-          <t>Hello,
-Are you tired of high commissions from Justdial or other directories?
-At Atrya Solutions, we build high-converting websites specifically for CCTV and electronic security companies like Home Security Direct.
-Our sites help you capture direct Google customers with instant 1-click WhatsApp quote buttons.
-See a DEMO of what we customize: https://atryasolutions.netlify.app/
-Would you be open to a quick 15-minute walkthrough to show you how we can boost your direct leads?
+          <t>Hi Home Security Direct Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -2827,7 +2940,7 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://wa.me/918478092778?text=Hi%20from%20Atrya%20Solutions%21%20%0A%0AWe%20help%20CCTV%20companies%20like%20Top%20Deal%20Trading%20get%20direct%20customers%20from%20Google%2C%20instead%20of%20relying%20on%20Justdial%20or%20social%20media.%20%0A%0AImagine%20a%20professional%20website%20with%20instant%20WhatsApp%20quotes.%20%0A%0ASee%20a%20DEMO%20of%20what%20we%20customize%3A%20https%3A//atryasolutions.netlify.app/%20%0A%0AWould%20you%20be%20open%20to%20a%2015-min%20walkthrough%3F</t>
+          <t>https://wa.me/918478092778?text=Hi%20Top%20Deal%20Trading%20-%20TV%205ALE%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr"/>
@@ -2905,25 +3018,33 @@
       <c r="AL14" s="2" t="inlineStr"/>
       <c r="AM14" s="2" t="inlineStr">
         <is>
-          <t>Hi from Atrya Solutions! 
-We help CCTV companies like Top Deal Trading get direct customers from Google, instead of relying on Justdial or social media. 
-Imagine a professional website with instant WhatsApp quotes. 
-See a DEMO of what we customize: https://atryasolutions.netlify.app/ 
-Would you be open to a 15-min walkthrough?</t>
+          <t>Hi Top Deal Trading - TV 5ALE,
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>Stop Paying Justdial Commissions?</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Top Deal Trading - TV 5ALE</t>
         </is>
       </c>
       <c r="AO14" s="2" t="inlineStr">
         <is>
-          <t>Hi Top Deal Trading,
-Are you tired of paying commissions to Justdial or limiting your reach to social media?
-At Atrya Solutions, we build high-converting websites specifically for CCTV companies. Our sites help you capture direct customers from Google with features like instant 1-click WhatsApp quote buttons.
-See a DEMO of what we customize: https://atryasolutions.netlify.app/
-Would you be open to a quick 15-minute walkthrough to show you how we can boost your direct enquiries?
+          <t>Hi Top Deal Trading - TV 5ALE Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -3012,7 +3133,7 @@
       </c>
       <c r="Q15" s="5" t="inlineStr">
         <is>
-          <t>https://wa.me/917892328427?text=Hi%20SKYWAY%20INFOSYSTEMS%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%20but%20doesn%27t%20have%20a%20direct%20website.%0AWe%20build%20websites%20and%20technician%20dispatch%20panels%20for%20CCTV%20installers.%0ACheck%20out%20our%20demo%3A%20https%3A//atryasolutions.netlify.app/%0AOpen%20for%20a%20quick%2010-min%20demo%3F</t>
+          <t>https://wa.me/917892328427?text=Hi%20SKYWAY%20INFOSYSTEMS%2C%0ANoticed%20your%20CCTV%20business%20in%2050%20gets%20great%20reviews%2C%20but%20you%20don%27t%20have%20a%20direct%20website%20yet%21%0A%0AYou%20might%20be%20losing%20direct%20Google%20customers%20or%20paying%20high%20commissions%20on%20Justdial.%20We%20build%20complete%20turnkey%20setups%20for%20CCTV%20companies%3A%0A%F0%9F%91%89%20Customer%20Website%20%281-Click%20WhatsApp%20Quotes%29%3A%20https%3A//atryasolutions.netlify.app/%0A%F0%9F%91%89%20Operations%20Admin%20%28Technician%20%26%20AMC%20Dispatch%29%3A%20https%3A//atryasolutions.netlify.app/admin%0A%0AOpen%20for%20a%20quick%2010-min%20walkthrough%20this%20week%3F</t>
         </is>
       </c>
       <c r="R15" s="4" t="inlineStr"/>
@@ -3083,24 +3204,32 @@
       <c r="AM15" s="4" t="inlineStr">
         <is>
           <t>Hi SKYWAY INFOSYSTEMS,
-Noticed your CCTV business in 50 gets great reviews but doesn't have a direct website.
-We build websites and technician dispatch panels for CCTV installers.
-Check out our demo: https://atryasolutions.netlify.app/
-Open for a quick 10-min demo?</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN15" s="4" t="inlineStr">
         <is>
-          <t>Direct website &amp; AMC panel for SKYWAY INFOSYSTEMS</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for SKYWAY INFOSYSTEMS</t>
         </is>
       </c>
       <c r="AO15" s="4" t="inlineStr">
         <is>
-          <t>Hi SKYWAY INFOSYSTEMS,
-I noticed you have strong customer reviews in 50, but potential clients searching Google might not find a direct website to request CCTV quotes.
-At Atrya Solutions, we set up turnkey websites with instant WhatsApp quote buttons and an operations panel to manage AMC maintenance contracts and field technicians.
-Live demo: https://atryasolutions.netlify.app/
-Would you be open to a 10-minute walkthrough this week?
+          <t>Hi SKYWAY INFOSYSTEMS Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>
@@ -3248,24 +3377,32 @@
       <c r="AM16" s="2" t="inlineStr">
         <is>
           <t>Hi Dynamic CCTV Ltd,
-Noticed your CCTV business in 50 gets great reviews but doesn't have a direct website.
-We build websites and technician dispatch panels for CCTV installers.
-Check out our demo: https://atryasolutions.netlify.app/
-Open for a quick 10-min demo?</t>
+Noticed your CCTV business in 50 gets great reviews, but you don't have a direct website yet!
+You might be losing direct Google customers or paying high commissions on Justdial. We build complete turnkey setups for CCTV companies:
+👉 Customer Website (1-Click WhatsApp Quotes): https://atryasolutions.netlify.app/
+👉 Operations Admin (Technician &amp; AMC Dispatch): https://atryasolutions.netlify.app/admin
+Open for a quick 10-min walkthrough this week?</t>
         </is>
       </c>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>Direct website &amp; AMC panel for Dynamic CCTV Ltd</t>
+          <t>Direct Customer Website &amp; AMC Admin Panel for Dynamic CCTV Ltd</t>
         </is>
       </c>
       <c r="AO16" s="2" t="inlineStr">
         <is>
-          <t>Hi Dynamic CCTV Ltd,
-I noticed you have strong customer reviews in 50, but potential clients searching Google might not find a direct website to request CCTV quotes.
-At Atrya Solutions, we set up turnkey websites with instant WhatsApp quote buttons and an operations panel to manage AMC maintenance contracts and field technicians.
-Live demo: https://atryasolutions.netlify.app/
-Would you be open to a 10-minute walkthrough this week?
+          <t>Hi Dynamic CCTV Ltd Team,
+I came across your CCTV business in 50 and saw your positive customer ratings. However, I noticed that potential clients searching Google cannot find a direct website to request CCTV quotes.
+Relying solely on local directories means you share leads with 4–5 competitors and pay ongoing commissions.
+At Atrya Solutions, we build complete turnkey systems specifically for CCTV and security installers:
+1. Customer-Facing Website (captures direct leads with 1-click WhatsApp quotes):
+   👉 Demo: https://atryasolutions.netlify.app/
+2. Operations Admin Panel (tracks jobs, AMC maintenance contracts, and technician dispatch):
+   👉 Demo Admin: https://atryasolutions.netlify.app/admin
+We customize and deliver the complete setup in 48 hours.
+Would you be open to a brief 10-minute walkthrough this week to see how this can grow your direct inquiries?
+Best regards,
+Atrya Solutions Team
 Reply STOP and I won't contact you again.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
chore: sync 58 enriched leads and updated leads_dashboard.html
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CCTV Leads" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCTV Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
@@ -742,7 +742,11 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>cid_3334184614186372508</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>PITCH_DRAFTED</t>
@@ -770,7 +774,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -4129,7 +4133,11 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>cid_13760439922089000441</t>
+        </is>
+      </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
           <t>PITCH_DRAFTED</t>
@@ -4157,7 +4165,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4320,7 +4328,11 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="4" t="inlineStr"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>cid_9009305908370015728</t>
+        </is>
+      </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
           <t>PITCH_DRAFTED</t>
@@ -4348,7 +4360,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr"/>
@@ -5101,7 +5113,11 @@
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="4" t="inlineStr"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>cid_15286622477168565426</t>
+        </is>
+      </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
           <t>PITCH_DRAFTED</t>
@@ -5129,7 +5145,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
@@ -5311,7 +5327,11 @@
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>cid_11514133238201629577</t>
+        </is>
+      </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
           <t>PITCH_DRAFTED</t>
@@ -5339,7 +5359,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Chintalkunta</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -6119,10 +6139,14 @@
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>cid_17997815080243066282</t>
+        </is>
+      </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -6147,7 +6171,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Keralam</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6271,9 +6295,30 @@
         </is>
       </c>
       <c r="AN30" s="2" t="inlineStr"/>
-      <c r="AO30" s="2" t="inlineStr"/>
-      <c r="AP30" s="2" t="inlineStr"/>
-      <c r="AQ30" s="2" t="inlineStr"/>
+      <c r="AO30" s="2" t="inlineStr">
+        <is>
+          <t>Hi Dahua wiki,
+Took a look at your CCTV website in Keralam and noticed a few things holding back customer enquiries (slow load time (6.0s); no direct WhatsApp contact widget).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP30" s="2" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for Dahua wiki</t>
+        </is>
+      </c>
+      <c r="AQ30" s="2" t="inlineStr">
+        <is>
+          <t>Hi Dahua wiki,
+I was looking up CCTV providers in Keralam and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: slow load time (6.0s); no direct WhatsApp contact widget.
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR30" s="2" t="inlineStr">
         <is>
           <t>2026-10-08 16:39:49</t>
@@ -6288,7 +6333,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -6367,7 +6412,11 @@
           <t>919110421987</t>
         </is>
       </c>
-      <c r="S31" s="4" t="inlineStr"/>
+      <c r="S31" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919110421987?text=Hi%20I%20Pro%20Secure%20CCTV%20CAMERA%20INSTALLATION%2C%0ATook%20a%20look%20at%20your%20CCTV%20website%20in%20Bengaluru%20and%20noticed%20a%20few%20things%20holding%20back%20customer%20enquiries%20%28no%20online%20enquiry%20or%20quote%20form%3B%20no%20direct%20WhatsApp%20contact%20widget%29.%0AWe%20build%20modern%20sites%20with%20instant%20WhatsApp%20quote%20buttons%3A%20https%3A//atryasolutions.netlify.app/%0AOpen%20to%20a%20quick%20demo%3F</t>
+        </is>
+      </c>
       <c r="T31" s="4" t="inlineStr"/>
       <c r="U31" s="4" t="inlineStr"/>
       <c r="V31" s="5" t="inlineStr">
@@ -6445,9 +6494,30 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO31" s="4" t="inlineStr"/>
-      <c r="AP31" s="4" t="inlineStr"/>
-      <c r="AQ31" s="4" t="inlineStr"/>
+      <c r="AO31" s="4" t="inlineStr">
+        <is>
+          <t>Hi I Pro Secure CCTV CAMERA INSTALLATION,
+Took a look at your CCTV website in Bengaluru and noticed a few things holding back customer enquiries (no online enquiry or quote form; no direct WhatsApp contact widget).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP31" s="4" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for I Pro Secure CCTV CAMERA INSTALLATION</t>
+        </is>
+      </c>
+      <c r="AQ31" s="4" t="inlineStr">
+        <is>
+          <t>Hi I Pro Secure CCTV CAMERA INSTALLATION,
+I was looking up CCTV providers in Bengaluru and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: no online enquiry or quote form; no direct WhatsApp contact widget.
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR31" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -6462,7 +6532,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -6541,7 +6611,11 @@
           <t>919741427427</t>
         </is>
       </c>
-      <c r="S32" s="2" t="inlineStr"/>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919741427427?text=Hi%20RAMESH%20CCTV%2C%0ATook%20a%20look%20at%20your%20CCTV%20website%20in%20Bengaluru%20and%20noticed%20a%20few%20things%20holding%20back%20customer%20enquiries%20%28no%20online%20enquiry%20or%20quote%20form%3B%20no%20direct%20WhatsApp%20contact%20widget%29.%0AWe%20build%20modern%20sites%20with%20instant%20WhatsApp%20quote%20buttons%3A%20https%3A//atryasolutions.netlify.app/%0AOpen%20to%20a%20quick%20demo%3F</t>
+        </is>
+      </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
           <t>6399999857; 6999999881; 7606708560</t>
@@ -6623,9 +6697,30 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="AO32" s="2" t="inlineStr"/>
-      <c r="AP32" s="2" t="inlineStr"/>
-      <c r="AQ32" s="2" t="inlineStr"/>
+      <c r="AO32" s="2" t="inlineStr">
+        <is>
+          <t>Hi RAMESH CCTV,
+Took a look at your CCTV website in Bengaluru and noticed a few things holding back customer enquiries (no online enquiry or quote form; no direct WhatsApp contact widget).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP32" s="2" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for RAMESH CCTV</t>
+        </is>
+      </c>
+      <c r="AQ32" s="2" t="inlineStr">
+        <is>
+          <t>Hi RAMESH CCTV,
+I was looking up CCTV providers in Bengaluru and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: no online enquiry or quote form; no direct WhatsApp contact widget.
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR32" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -6640,7 +6735,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -6719,7 +6814,11 @@
           <t>919035080007</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr"/>
+      <c r="S33" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919035080007?text=Hi%20SIXAXIS%20CCTV%2C%0ATook%20a%20look%20at%20your%20CCTV%20website%20in%20Bengaluru%20and%20noticed%20a%20few%20things%20holding%20back%20customer%20enquiries%20%28not%20served%20over%20HTTPS%20%28insecure%20connection%29%29.%0AWe%20build%20modern%20sites%20with%20instant%20WhatsApp%20quote%20buttons%3A%20https%3A//atryasolutions.netlify.app/%0AOpen%20to%20a%20quick%20demo%3F</t>
+        </is>
+      </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
           <t>+919035030007</t>
@@ -6821,9 +6920,30 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO33" s="4" t="inlineStr"/>
-      <c r="AP33" s="4" t="inlineStr"/>
-      <c r="AQ33" s="4" t="inlineStr"/>
+      <c r="AO33" s="4" t="inlineStr">
+        <is>
+          <t>Hi SIXAXIS CCTV,
+Took a look at your CCTV website in Bengaluru and noticed a few things holding back customer enquiries (not served over HTTPS (insecure connection)).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP33" s="4" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for SIXAXIS CCTV</t>
+        </is>
+      </c>
+      <c r="AQ33" s="4" t="inlineStr">
+        <is>
+          <t>Hi SIXAXIS CCTV,
+I was looking up CCTV providers in Bengaluru and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: not served over HTTPS (insecure connection).
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR33" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -6838,7 +6958,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -6917,7 +7037,11 @@
           <t>919538380555</t>
         </is>
       </c>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919538380555?text=Hi%20CCTV%20SHOPPING%2C%0ATook%20a%20look%20at%20your%20CCTV%20website%20in%20Bengaluru%20and%20noticed%20a%20few%20things%20holding%20back%20customer%20enquiries%20%28no%20online%20enquiry%20or%20quote%20form%3B%20no%20direct%20WhatsApp%20contact%20widget%29.%0AWe%20build%20modern%20sites%20with%20instant%20WhatsApp%20quote%20buttons%3A%20https%3A//atryasolutions.netlify.app/%0AOpen%20to%20a%20quick%20demo%3F</t>
+        </is>
+      </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
           <t>+919538380555; 6395939088; 6666666667</t>
@@ -6999,9 +7123,30 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="AO34" s="2" t="inlineStr"/>
-      <c r="AP34" s="2" t="inlineStr"/>
-      <c r="AQ34" s="2" t="inlineStr"/>
+      <c r="AO34" s="2" t="inlineStr">
+        <is>
+          <t>Hi CCTV SHOPPING,
+Took a look at your CCTV website in Bengaluru and noticed a few things holding back customer enquiries (no online enquiry or quote form; no direct WhatsApp contact widget).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP34" s="2" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for CCTV SHOPPING</t>
+        </is>
+      </c>
+      <c r="AQ34" s="2" t="inlineStr">
+        <is>
+          <t>Hi CCTV SHOPPING,
+I was looking up CCTV providers in Bengaluru and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: no online enquiry or quote form; no direct WhatsApp contact widget.
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR34" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -7016,7 +7161,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -7095,7 +7240,11 @@
           <t>919739933180</t>
         </is>
       </c>
-      <c r="S35" s="4" t="inlineStr"/>
+      <c r="S35" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919739933180?text=Hi%20KWALITY%20TECH%20ZONE%20LLP%2C%0ATook%20a%20look%20at%20your%20CCTV%20website%20in%20Bengaluru%20and%20noticed%20a%20few%20things%20holding%20back%20customer%20enquiries%20%28no%20online%20enquiry%20or%20quote%20form%3B%20no%20direct%20WhatsApp%20contact%20widget%29.%0AWe%20build%20modern%20sites%20with%20instant%20WhatsApp%20quote%20buttons%3A%20https%3A//atryasolutions.netlify.app/%0AOpen%20to%20a%20quick%20demo%3F</t>
+        </is>
+      </c>
       <c r="T35" s="4" t="inlineStr"/>
       <c r="U35" s="4" t="inlineStr"/>
       <c r="V35" s="5" t="inlineStr">
@@ -7169,9 +7318,30 @@
         </is>
       </c>
       <c r="AN35" s="4" t="inlineStr"/>
-      <c r="AO35" s="4" t="inlineStr"/>
-      <c r="AP35" s="4" t="inlineStr"/>
-      <c r="AQ35" s="4" t="inlineStr"/>
+      <c r="AO35" s="4" t="inlineStr">
+        <is>
+          <t>Hi KWALITY TECH ZONE LLP,
+Took a look at your CCTV website in Bengaluru and noticed a few things holding back customer enquiries (no online enquiry or quote form; no direct WhatsApp contact widget).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP35" s="4" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for KWALITY TECH ZONE LLP</t>
+        </is>
+      </c>
+      <c r="AQ35" s="4" t="inlineStr">
+        <is>
+          <t>Hi KWALITY TECH ZONE LLP,
+I was looking up CCTV providers in Bengaluru and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: no online enquiry or quote form; no direct WhatsApp contact widget.
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR35" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:56</t>
@@ -7186,7 +7356,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -7335,9 +7505,30 @@
         </is>
       </c>
       <c r="AN36" s="2" t="inlineStr"/>
-      <c r="AO36" s="2" t="inlineStr"/>
-      <c r="AP36" s="2" t="inlineStr"/>
-      <c r="AQ36" s="2" t="inlineStr"/>
+      <c r="AO36" s="2" t="inlineStr">
+        <is>
+          <t>Hi Bangalore Electronics,
+Took a look at your CCTV website in Bengaluru and noticed a few things holding back customer enquiries (no online enquiry or quote form; no direct WhatsApp contact widget).
+We build modern sites with instant WhatsApp quote buttons: https://atryasolutions.netlify.app/
+Open to a quick demo?</t>
+        </is>
+      </c>
+      <c r="AP36" s="2" t="inlineStr">
+        <is>
+          <t>Improving CCTV quote enquiries for Bangalore Electronics</t>
+        </is>
+      </c>
+      <c r="AQ36" s="2" t="inlineStr">
+        <is>
+          <t>Hi Bangalore Electronics,
+I was looking up CCTV providers in Bengaluru and checked your website.
+I noticed a couple of areas that might be reducing your lead conversion: no online enquiry or quote form; no direct WhatsApp contact widget.
+At Atrya Solutions, we build high-converting websites and AMC management systems for security installers.
+Live demo: https://atryasolutions.netlify.app/
+Would you be interested in a brief 10-minute walkthrough?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR36" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:57</t>
@@ -7345,10 +7536,14 @@
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="4" t="inlineStr"/>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>cid_12014290968981143054</t>
+        </is>
+      </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -7373,7 +7568,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
@@ -7427,7 +7622,11 @@
           <t>919738966594</t>
         </is>
       </c>
-      <c r="S37" s="4" t="inlineStr"/>
+      <c r="S37" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919738966594?text=Hi%20Cyber%20Pro%20India%20-%20CCTV%20Installation%20Service%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
           <t>+91-9738966594; +919738966594; 6062210545</t>
@@ -7529,9 +7728,29 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="AO37" s="4" t="inlineStr"/>
-      <c r="AP37" s="4" t="inlineStr"/>
-      <c r="AQ37" s="4" t="inlineStr"/>
+      <c r="AO37" s="4" t="inlineStr">
+        <is>
+          <t>Hi Cyber Pro India - CCTV Installation Service,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP37" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Cyber Pro India - CCTV Installation Service</t>
+        </is>
+      </c>
+      <c r="AQ37" s="4" t="inlineStr">
+        <is>
+          <t>Hi Cyber Pro India - CCTV Installation Service,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR37" s="4" t="inlineStr">
         <is>
           <t>2026-10-08 16:39:44</t>
@@ -7546,7 +7765,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7625,7 +7844,11 @@
           <t>919686550099</t>
         </is>
       </c>
-      <c r="S38" s="2" t="inlineStr"/>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919686550099?text=Hi%20Skafoss%20Technologies%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
           <t>+919686550099; 6283185841; 9308893008</t>
@@ -7711,9 +7934,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO38" s="2" t="inlineStr"/>
-      <c r="AP38" s="2" t="inlineStr"/>
-      <c r="AQ38" s="2" t="inlineStr"/>
+      <c r="AO38" s="2" t="inlineStr">
+        <is>
+          <t>Hi Skafoss Technologies,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP38" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Skafoss Technologies</t>
+        </is>
+      </c>
+      <c r="AQ38" s="2" t="inlineStr">
+        <is>
+          <t>Hi Skafoss Technologies,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR38" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -7728,7 +7971,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -7807,7 +8050,11 @@
           <t>919620421001</t>
         </is>
       </c>
-      <c r="S39" s="4" t="inlineStr"/>
+      <c r="S39" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919620421001?text=Hi%20KING%20TECHNOLOGY%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
           <t>+919019390194; +919620421001; 6207859085</t>
@@ -7893,9 +8140,29 @@
         </is>
       </c>
       <c r="AN39" s="4" t="inlineStr"/>
-      <c r="AO39" s="4" t="inlineStr"/>
-      <c r="AP39" s="4" t="inlineStr"/>
-      <c r="AQ39" s="4" t="inlineStr"/>
+      <c r="AO39" s="4" t="inlineStr">
+        <is>
+          <t>Hi KING TECHNOLOGY,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP39" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for KING TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="AQ39" s="4" t="inlineStr">
+        <is>
+          <t>Hi KING TECHNOLOGY,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR39" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -7910,7 +8177,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -7989,7 +8256,11 @@
           <t>918147148767</t>
         </is>
       </c>
-      <c r="S40" s="2" t="inlineStr"/>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/918147148767?text=Hi%20MY%20DISTRIBUTOR%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T40" s="2" t="inlineStr">
         <is>
           <t>6281040558</t>
@@ -8083,9 +8354,29 @@
         </is>
       </c>
       <c r="AN40" s="2" t="inlineStr"/>
-      <c r="AO40" s="2" t="inlineStr"/>
-      <c r="AP40" s="2" t="inlineStr"/>
-      <c r="AQ40" s="2" t="inlineStr"/>
+      <c r="AO40" s="2" t="inlineStr">
+        <is>
+          <t>Hi MY DISTRIBUTOR,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP40" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for MY DISTRIBUTOR</t>
+        </is>
+      </c>
+      <c r="AQ40" s="2" t="inlineStr">
+        <is>
+          <t>Hi MY DISTRIBUTOR,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR40" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:55</t>
@@ -8100,7 +8391,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -8179,7 +8470,11 @@
           <t>919513533180</t>
         </is>
       </c>
-      <c r="S41" s="4" t="inlineStr"/>
+      <c r="S41" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919513533180?text=Hi%20CAMERA%20COUNTRY%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
           <t>+91-9513533180; +919513533180; 9513533180</t>
@@ -8273,9 +8568,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO41" s="4" t="inlineStr"/>
-      <c r="AP41" s="4" t="inlineStr"/>
-      <c r="AQ41" s="4" t="inlineStr"/>
+      <c r="AO41" s="4" t="inlineStr">
+        <is>
+          <t>Hi CAMERA COUNTRY,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP41" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for CAMERA COUNTRY</t>
+        </is>
+      </c>
+      <c r="AQ41" s="4" t="inlineStr">
+        <is>
+          <t>Hi CAMERA COUNTRY,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR41" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:57</t>
@@ -8290,7 +8605,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -8369,7 +8684,11 @@
           <t>917353033399</t>
         </is>
       </c>
-      <c r="S42" s="2" t="inlineStr"/>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/917353033399?text=Hi%20Star%20vision%20solutions%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T42" s="2" t="inlineStr">
         <is>
           <t>+91 7353033399; +91 7892988076; 7353033399</t>
@@ -8455,9 +8774,29 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="AO42" s="2" t="inlineStr"/>
-      <c r="AP42" s="2" t="inlineStr"/>
-      <c r="AQ42" s="2" t="inlineStr"/>
+      <c r="AO42" s="2" t="inlineStr">
+        <is>
+          <t>Hi Star vision solutions,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP42" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Star vision solutions</t>
+        </is>
+      </c>
+      <c r="AQ42" s="2" t="inlineStr">
+        <is>
+          <t>Hi Star vision solutions,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR42" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -8472,7 +8811,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -8621,9 +8960,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO43" s="4" t="inlineStr"/>
-      <c r="AP43" s="4" t="inlineStr"/>
-      <c r="AQ43" s="4" t="inlineStr"/>
+      <c r="AO43" s="4" t="inlineStr">
+        <is>
+          <t>Hi VISION ZOOM SECURITY SYSTEMS,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP43" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for VISION ZOOM SECURITY SYSTEMS</t>
+        </is>
+      </c>
+      <c r="AQ43" s="4" t="inlineStr">
+        <is>
+          <t>Hi VISION ZOOM SECURITY SYSTEMS,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR43" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:55</t>
@@ -8638,7 +8997,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -8717,7 +9076,11 @@
           <t>919686037552</t>
         </is>
       </c>
-      <c r="S44" s="2" t="inlineStr"/>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919686037552?text=Hi%20HM%20Security%20Solutions%20%28CCTV%20Sales%20%26%20Service%29%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T44" s="2" t="inlineStr">
         <is>
           <t>6616527297; 6771901355; 9686037552</t>
@@ -8799,9 +9162,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO44" s="2" t="inlineStr"/>
-      <c r="AP44" s="2" t="inlineStr"/>
-      <c r="AQ44" s="2" t="inlineStr"/>
+      <c r="AO44" s="2" t="inlineStr">
+        <is>
+          <t>Hi HM Security Solutions (CCTV Sales &amp; Service),
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP44" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for HM Security Solutions (CCTV Sales &amp; Service)</t>
+        </is>
+      </c>
+      <c r="AQ44" s="2" t="inlineStr">
+        <is>
+          <t>Hi HM Security Solutions (CCTV Sales &amp; Service),
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR44" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -8816,7 +9199,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -8895,7 +9278,11 @@
           <t>918618084202</t>
         </is>
       </c>
-      <c r="S45" s="4" t="inlineStr"/>
+      <c r="S45" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/918618084202?text=Hi%20Bangalore%20It%20Hub%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
           <t>+91 8618084202; +918618084202; 6215384432</t>
@@ -8977,9 +9364,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO45" s="4" t="inlineStr"/>
-      <c r="AP45" s="4" t="inlineStr"/>
-      <c r="AQ45" s="4" t="inlineStr"/>
+      <c r="AO45" s="4" t="inlineStr">
+        <is>
+          <t>Hi Bangalore It Hub,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP45" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Bangalore It Hub</t>
+        </is>
+      </c>
+      <c r="AQ45" s="4" t="inlineStr">
+        <is>
+          <t>Hi Bangalore It Hub,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR45" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:55</t>
@@ -8994,7 +9401,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -9073,7 +9480,11 @@
           <t>918618682725</t>
         </is>
       </c>
-      <c r="S46" s="2" t="inlineStr"/>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/918618682725?text=Hi%20Mayur%20Infotech%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T46" s="2" t="inlineStr">
         <is>
           <t>+918618682725; 8011444930; 8618682725</t>
@@ -9155,9 +9566,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO46" s="2" t="inlineStr"/>
-      <c r="AP46" s="2" t="inlineStr"/>
-      <c r="AQ46" s="2" t="inlineStr"/>
+      <c r="AO46" s="2" t="inlineStr">
+        <is>
+          <t>Hi Mayur Infotech,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP46" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Mayur Infotech</t>
+        </is>
+      </c>
+      <c r="AQ46" s="2" t="inlineStr">
+        <is>
+          <t>Hi Mayur Infotech,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR46" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:56</t>
@@ -9172,7 +9603,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -9251,7 +9682,11 @@
           <t>919916161100</t>
         </is>
       </c>
-      <c r="S47" s="4" t="inlineStr"/>
+      <c r="S47" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919916161100?text=Hi%20Rajlaxmi%20infotech%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
           <t>+91 9916161100; +919916161100</t>
@@ -9333,9 +9768,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO47" s="4" t="inlineStr"/>
-      <c r="AP47" s="4" t="inlineStr"/>
-      <c r="AQ47" s="4" t="inlineStr"/>
+      <c r="AO47" s="4" t="inlineStr">
+        <is>
+          <t>Hi Rajlaxmi infotech,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP47" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Rajlaxmi infotech</t>
+        </is>
+      </c>
+      <c r="AQ47" s="4" t="inlineStr">
+        <is>
+          <t>Hi Rajlaxmi infotech,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR47" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:57</t>
@@ -9343,10 +9798,14 @@
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="2" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>cid_16943958218051604871</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -9371,7 +9830,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Zirakpur</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9425,7 +9884,11 @@
           <t>916239110669</t>
         </is>
       </c>
-      <c r="S48" s="2" t="inlineStr"/>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/916239110669?text=Hi%20Web%20Plus%20Security%20System%2C%0ASaw%20your%20CCTV%20website%20in%20Zirakpur.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T48" s="2" t="inlineStr">
         <is>
           <t>+91 9115704767; 9115704767; 9467284332</t>
@@ -9507,9 +9970,29 @@
         </is>
       </c>
       <c r="AN48" s="2" t="inlineStr"/>
-      <c r="AO48" s="2" t="inlineStr"/>
-      <c r="AP48" s="2" t="inlineStr"/>
-      <c r="AQ48" s="2" t="inlineStr"/>
+      <c r="AO48" s="2" t="inlineStr">
+        <is>
+          <t>Hi Web Plus Security System,
+Saw your CCTV website in Zirakpur. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP48" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Web Plus Security System</t>
+        </is>
+      </c>
+      <c r="AQ48" s="2" t="inlineStr">
+        <is>
+          <t>Hi Web Plus Security System,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR48" s="2" t="inlineStr">
         <is>
           <t>2026-10-08 16:39:53</t>
@@ -9524,7 +10007,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -9603,7 +10086,11 @@
           <t>919035362143</t>
         </is>
       </c>
-      <c r="S49" s="4" t="inlineStr"/>
+      <c r="S49" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919035362143?text=Hi%20Yendra%20Techno%20Solution%20-%20CCTV%20Cameras%20Installation%20in%20Bengaluru%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T49" s="4" t="inlineStr">
         <is>
           <t>+919035362143; +919353316120</t>
@@ -9685,9 +10172,29 @@
         </is>
       </c>
       <c r="AN49" s="4" t="inlineStr"/>
-      <c r="AO49" s="4" t="inlineStr"/>
-      <c r="AP49" s="4" t="inlineStr"/>
-      <c r="AQ49" s="4" t="inlineStr"/>
+      <c r="AO49" s="4" t="inlineStr">
+        <is>
+          <t>Hi Yendra Techno Solution - CCTV Cameras Installation in Bengaluru,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP49" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Yendra Techno Solution - CCTV Cameras Installation in Bengaluru</t>
+        </is>
+      </c>
+      <c r="AQ49" s="4" t="inlineStr">
+        <is>
+          <t>Hi Yendra Techno Solution - CCTV Cameras Installation in Bengaluru,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR49" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -9702,7 +10209,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -9781,7 +10288,11 @@
           <t>916361264243</t>
         </is>
       </c>
-      <c r="S50" s="2" t="inlineStr"/>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/916361264243?text=Hi%20CCTV%20Surveillance%20Cameras%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T50" s="2" t="inlineStr">
         <is>
           <t>+916361264243; 6060429773; 6361264243</t>
@@ -9871,9 +10382,29 @@
         </is>
       </c>
       <c r="AN50" s="2" t="inlineStr"/>
-      <c r="AO50" s="2" t="inlineStr"/>
-      <c r="AP50" s="2" t="inlineStr"/>
-      <c r="AQ50" s="2" t="inlineStr"/>
+      <c r="AO50" s="2" t="inlineStr">
+        <is>
+          <t>Hi CCTV Surveillance Cameras,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP50" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for CCTV Surveillance Cameras</t>
+        </is>
+      </c>
+      <c r="AQ50" s="2" t="inlineStr">
+        <is>
+          <t>Hi CCTV Surveillance Cameras,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR50" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -9888,7 +10419,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -10045,9 +10576,29 @@
         </is>
       </c>
       <c r="AN51" s="4" t="inlineStr"/>
-      <c r="AO51" s="4" t="inlineStr"/>
-      <c r="AP51" s="4" t="inlineStr"/>
-      <c r="AQ51" s="4" t="inlineStr"/>
+      <c r="AO51" s="4" t="inlineStr">
+        <is>
+          <t>Hi MY COMPUTER AND CCTV ZONE,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP51" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for MY COMPUTER AND CCTV ZONE</t>
+        </is>
+      </c>
+      <c r="AQ51" s="4" t="inlineStr">
+        <is>
+          <t>Hi MY COMPUTER AND CCTV ZONE,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR51" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -10062,7 +10613,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -10141,7 +10692,11 @@
           <t>917026113516</t>
         </is>
       </c>
-      <c r="S52" s="2" t="inlineStr"/>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/917026113516?text=Hi%20i2secure%20%E2%80%93%20Smart%20CCTV%20Solutions%20Bengaluru%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T52" s="2" t="inlineStr">
         <is>
           <t>+917026113516; 7026113516</t>
@@ -10219,9 +10774,29 @@
         </is>
       </c>
       <c r="AN52" s="2" t="inlineStr"/>
-      <c r="AO52" s="2" t="inlineStr"/>
-      <c r="AP52" s="2" t="inlineStr"/>
-      <c r="AQ52" s="2" t="inlineStr"/>
+      <c r="AO52" s="2" t="inlineStr">
+        <is>
+          <t>Hi i2secure – Smart CCTV Solutions Bengaluru,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP52" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for i2secure – Smart CCTV Solutions Bengaluru</t>
+        </is>
+      </c>
+      <c r="AQ52" s="2" t="inlineStr">
+        <is>
+          <t>Hi i2secure – Smart CCTV Solutions Bengaluru,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR52" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -10236,7 +10811,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -10315,7 +10890,11 @@
           <t>918660317664</t>
         </is>
       </c>
-      <c r="S53" s="4" t="inlineStr"/>
+      <c r="S53" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/918660317664?text=Hi%20Agasthya%20Electronics%20%7C%20CCTV%2C%20Solar%20Sim%20Cameras%2C%20Wi-Fi%20Cameras%2C%20Digital%20Door%20Locks%2C%20Video%20Door%20Phones%2C%20Access%20Control%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T53" s="4" t="inlineStr">
         <is>
           <t>8660317664; 9096313912</t>
@@ -10417,9 +10996,29 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="AO53" s="4" t="inlineStr"/>
-      <c r="AP53" s="4" t="inlineStr"/>
-      <c r="AQ53" s="4" t="inlineStr"/>
+      <c r="AO53" s="4" t="inlineStr">
+        <is>
+          <t>Hi Agasthya Electronics | CCTV, Solar Sim Cameras, Wi-Fi Cameras, Digital Door Locks, Video Door Phones, Access Control,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP53" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Agasthya Electronics | CCTV, Solar Sim Cameras, Wi-Fi Cameras, Digital Door Locks, Video Door Phones, Access Control</t>
+        </is>
+      </c>
+      <c r="AQ53" s="4" t="inlineStr">
+        <is>
+          <t>Hi Agasthya Electronics | CCTV, Solar Sim Cameras, Wi-Fi Cameras, Digital Door Locks, Video Door Phones, Access Control,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR53" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:56</t>
@@ -10434,7 +11033,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -10513,7 +11112,11 @@
           <t>919902234508</t>
         </is>
       </c>
-      <c r="S54" s="2" t="inlineStr"/>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919902234508?text=Hi%20CCTV%20ZONE%20IN%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T54" s="2" t="inlineStr">
         <is>
           <t>+919902234508; 9902234508</t>
@@ -10591,9 +11194,29 @@
         </is>
       </c>
       <c r="AN54" s="2" t="inlineStr"/>
-      <c r="AO54" s="2" t="inlineStr"/>
-      <c r="AP54" s="2" t="inlineStr"/>
-      <c r="AQ54" s="2" t="inlineStr"/>
+      <c r="AO54" s="2" t="inlineStr">
+        <is>
+          <t>Hi CCTV ZONE IN,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP54" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for CCTV ZONE IN</t>
+        </is>
+      </c>
+      <c r="AQ54" s="2" t="inlineStr">
+        <is>
+          <t>Hi CCTV ZONE IN,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR54" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -10608,7 +11231,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -10687,7 +11310,11 @@
           <t>919980040399</t>
         </is>
       </c>
-      <c r="S55" s="4" t="inlineStr"/>
+      <c r="S55" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919980040399?text=Hi%20MYF%20CCTV%20%26%20security%20systems%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T55" s="4" t="inlineStr">
         <is>
           <t>+91 9980040399; +919980040399; 9980040399</t>
@@ -10769,9 +11396,29 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AO55" s="4" t="inlineStr"/>
-      <c r="AP55" s="4" t="inlineStr"/>
-      <c r="AQ55" s="4" t="inlineStr"/>
+      <c r="AO55" s="4" t="inlineStr">
+        <is>
+          <t>Hi MYF CCTV &amp; security systems,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP55" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for MYF CCTV &amp; security systems</t>
+        </is>
+      </c>
+      <c r="AQ55" s="4" t="inlineStr">
+        <is>
+          <t>Hi MYF CCTV &amp; security systems,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR55" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -10786,7 +11433,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -10865,7 +11512,11 @@
           <t>919739661248</t>
         </is>
       </c>
-      <c r="S56" s="2" t="inlineStr"/>
+      <c r="S56" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919739661248?text=Hi%20Computer%20IT%20Mart%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T56" s="2" t="inlineStr">
         <is>
           <t>+91 9620554635; +91 9739661248; 6267352236</t>
@@ -10959,9 +11610,29 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="AO56" s="2" t="inlineStr"/>
-      <c r="AP56" s="2" t="inlineStr"/>
-      <c r="AQ56" s="2" t="inlineStr"/>
+      <c r="AO56" s="2" t="inlineStr">
+        <is>
+          <t>Hi Computer IT Mart,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP56" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Computer IT Mart</t>
+        </is>
+      </c>
+      <c r="AQ56" s="2" t="inlineStr">
+        <is>
+          <t>Hi Computer IT Mart,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR56" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:56</t>
@@ -10976,7 +11647,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -11055,7 +11726,11 @@
           <t>917676954748</t>
         </is>
       </c>
-      <c r="S57" s="4" t="inlineStr"/>
+      <c r="S57" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/917676954748?text=Hi%20Anvi%20Tech%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T57" s="4" t="inlineStr"/>
       <c r="U57" s="4" t="inlineStr">
         <is>
@@ -11129,9 +11804,29 @@
         </is>
       </c>
       <c r="AN57" s="4" t="inlineStr"/>
-      <c r="AO57" s="4" t="inlineStr"/>
-      <c r="AP57" s="4" t="inlineStr"/>
-      <c r="AQ57" s="4" t="inlineStr"/>
+      <c r="AO57" s="4" t="inlineStr">
+        <is>
+          <t>Hi Anvi Tech,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP57" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for Anvi Tech</t>
+        </is>
+      </c>
+      <c r="AQ57" s="4" t="inlineStr">
+        <is>
+          <t>Hi Anvi Tech,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR57" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -11146,7 +11841,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -11225,7 +11920,11 @@
           <t>919353356153</t>
         </is>
       </c>
-      <c r="S58" s="2" t="inlineStr"/>
+      <c r="S58" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919353356153?text=Hi%20V-Tech%20-%20cctv%20cameras%20and%20installation%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
           <t>+919353356153; 7899999999</t>
@@ -11303,9 +12002,29 @@
         </is>
       </c>
       <c r="AN58" s="2" t="inlineStr"/>
-      <c r="AO58" s="2" t="inlineStr"/>
-      <c r="AP58" s="2" t="inlineStr"/>
-      <c r="AQ58" s="2" t="inlineStr"/>
+      <c r="AO58" s="2" t="inlineStr">
+        <is>
+          <t>Hi V-Tech - cctv cameras and installation,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP58" s="2" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for V-Tech - cctv cameras and installation</t>
+        </is>
+      </c>
+      <c r="AQ58" s="2" t="inlineStr">
+        <is>
+          <t>Hi V-Tech - cctv cameras and installation,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR58" s="2" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:55</t>
@@ -11320,7 +12039,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>PITCH_DRAFTED</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -11399,7 +12118,11 @@
           <t>919206979799</t>
         </is>
       </c>
-      <c r="S59" s="4" t="inlineStr"/>
+      <c r="S59" s="5" t="inlineStr">
+        <is>
+          <t>https://wa.me/919206979799?text=Hi%20CCTV%20Shield%20Care%2C%0ASaw%20your%20CCTV%20website%20in%20Bengaluru.%20How%20do%20you%20currently%20manage%20your%20AMC%20service%20renewals%20and%20technician%20dispatch%3F%0AWe%20built%20an%20operations%20panel%20specifically%20for%20security%20installers%3A%20https%3A//atryasolutions.netlify.app/admin%0AWorth%20a%20quick%20look%3F</t>
+        </is>
+      </c>
       <c r="T59" s="4" t="inlineStr">
         <is>
           <t>+919449776044; 6564498876; 9449776044</t>
@@ -11481,9 +12204,29 @@
         </is>
       </c>
       <c r="AN59" s="4" t="inlineStr"/>
-      <c r="AO59" s="4" t="inlineStr"/>
-      <c r="AP59" s="4" t="inlineStr"/>
-      <c r="AQ59" s="4" t="inlineStr"/>
+      <c r="AO59" s="4" t="inlineStr">
+        <is>
+          <t>Hi CCTV Shield Care,
+Saw your CCTV website in Bengaluru. How do you currently manage your AMC service renewals and technician dispatch?
+We built an operations panel specifically for security installers: https://atryasolutions.netlify.app/admin
+Worth a quick look?</t>
+        </is>
+      </c>
+      <c r="AP59" s="4" t="inlineStr">
+        <is>
+          <t>AMC tracking &amp; technician panel for CCTV Shield Care</t>
+        </is>
+      </c>
+      <c r="AQ59" s="4" t="inlineStr">
+        <is>
+          <t>Hi CCTV Shield Care,
+I came across your website and wanted to reach out.
+Most CCTV dealers tell us tracking annual maintenance contracts (AMCs), technician visits, and warranty renewals becomes chaotic on spreadsheets.
+We built a specialized operations panel for CCTV teams: https://atryasolutions.netlify.app/admin
+Would you be open to a quick 10-minute walkthrough to see if it saves your team time?
+Reply STOP and I won't contact you again.</t>
+        </is>
+      </c>
       <c r="AR59" s="4" t="inlineStr">
         <is>
           <t>2026-10-10 09:50:54</t>
@@ -11566,95 +12309,121 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V30" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V32" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V33" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y33" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA33" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V34" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V35" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V36" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V37" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y37" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V38" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V39" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V40" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V41" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V42" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V43" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V44" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V45" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V46" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V47" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V48" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X48" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V49" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V50" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V51" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X51" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V52" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V53" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X53" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V54" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V55" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V56" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X56" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V57" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V58" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V59" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X59" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V32" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V33" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y33" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA33" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V34" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V35" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V36" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V37" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y37" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V41" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V42" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V43" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V44" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V47" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V50" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V51" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X51" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S52" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V52" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S53" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V53" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X53" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S54" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V54" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S55" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V55" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S56" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V56" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X56" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S57" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V57" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S58" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V58" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S59" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V59" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X59" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId189"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>